<commit_message>
Refresh door notice PDF with revised rules
</commit_message>
<xml_diff>
--- a/2608_Inventary_List_Taekwang.xlsx
+++ b/2608_Inventary_List_Taekwang.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kwettstei\Nextcloud\Jang\Finance\Procurement\Various\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seung/Desktop/sk/ETHZ/EECIS/group_works/eecis-device-rental/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{110787A6-A4F8-44AB-9FFD-6982B647A540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24360" yWindow="3870" windowWidth="21600" windowHeight="12525" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -470,7 +470,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -486,7 +486,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -803,7 +803,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
@@ -816,7 +816,7 @@
     <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -845,7 +845,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -874,7 +874,7 @@
         <v>35475</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
@@ -903,7 +903,7 @@
         <v>35584</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
@@ -932,7 +932,7 @@
         <v>40900</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>29</v>
       </c>
@@ -961,7 +961,7 @@
         <v>43731</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
@@ -990,7 +990,7 @@
         <v>43731</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>38</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>43731</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>43</v>
       </c>
@@ -1048,7 +1048,7 @@
         <v>43762</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>49</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>43763</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>55</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>43969</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>61</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>43969</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>66</v>
       </c>
@@ -1164,7 +1164,7 @@
         <v>43969</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>71</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>43969</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>76</v>
       </c>
@@ -1222,7 +1222,7 @@
         <v>44455</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>81</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>44455</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>86</v>
       </c>
@@ -1280,7 +1280,7 @@
         <v>44902</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>91</v>
       </c>
@@ -1309,7 +1309,7 @@
         <v>45337</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>96</v>
       </c>
@@ -1336,7 +1336,7 @@
         <v>45782</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>100</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>45820</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>105</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>45820</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>110</v>
       </c>
@@ -1417,7 +1417,7 @@
         <v>45848</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>114</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>45876</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>119</v>
       </c>
@@ -1467,7 +1467,7 @@
         <v>45953</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>122</v>
       </c>
@@ -1492,7 +1492,7 @@
         <v>46000</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>126</v>
       </c>

</xml_diff>